<commit_message>
Limita propuesta de puestos solo a Valladolid
</commit_message>
<xml_diff>
--- a/data/kennedy_mira_consolidado.xlsx
+++ b/data/kennedy_mira_consolidado.xlsx
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>El tablero identifica 30 puestos de prioridad alta y 43 puestos con cambio operativo de templo sugerido, manteniendo separada la iglesia histórica 2026 del templo propuesto para operación territorial.</t>
+          <t>El tablero identifica 30 puestos de prioridad alta y 26 puestos con cambio operativo de templo sugerido, manteniendo separada la iglesia histórica 2026 del templo propuesto para operación territorial.</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como CARVAJAL.</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>PATIO BONITO</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K13" t="n">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: PATIO BONITO.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K20" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CLASS ROMA</t>
         </is>
       </c>
       <c r="K26" t="n">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K31" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="K32" t="n">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K33" t="n">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3753,7 +3753,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3909,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4143,7 +4143,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4299,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K45" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4689,7 +4689,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5157,7 +5157,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5313,7 +5313,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5391,7 +5391,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5585,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K59" t="n">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K61" t="n">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5859,7 +5859,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5937,7 +5937,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K64" t="n">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6053,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K65" t="n">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6249,7 @@
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -6405,7 +6405,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -6483,7 +6483,7 @@
       </c>
       <c r="V70" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6639,7 @@
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -6717,7 +6717,7 @@
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -6795,7 +6795,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -6951,7 +6951,7 @@
       </c>
       <c r="V76" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7029,7 @@
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="V78" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
     </row>
@@ -7185,7 +7185,7 @@
       </c>
       <c r="V79" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="K80" t="n">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7341,7 +7341,7 @@
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7419,7 +7419,7 @@
       </c>
       <c r="V82" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7497,7 +7497,7 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -7653,7 +7653,7 @@
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7731,7 +7731,7 @@
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7809,7 +7809,7 @@
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7847,7 +7847,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="K88" t="n">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="V89" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -8043,7 +8043,7 @@
       </c>
       <c r="V90" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="V91" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8199,7 +8199,7 @@
       </c>
       <c r="V92" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8355,7 +8355,7 @@
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8471,7 +8471,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K96" t="n">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8589,7 +8589,7 @@
       </c>
       <c r="V97" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -8627,7 +8627,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K98" t="n">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8745,7 +8745,7 @@
       </c>
       <c r="V99" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="V100" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
     </row>
@@ -8901,7 +8901,7 @@
       </c>
       <c r="V101" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -8979,7 +8979,7 @@
       </c>
       <c r="V102" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9057,7 +9057,7 @@
       </c>
       <c r="V103" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9135,7 +9135,7 @@
       </c>
       <c r="V104" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -9213,7 +9213,7 @@
       </c>
       <c r="V105" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9291,7 +9291,7 @@
       </c>
       <c r="V106" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="V107" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9447,7 +9447,7 @@
       </c>
       <c r="V108" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9525,7 +9525,7 @@
       </c>
       <c r="V109" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9603,7 +9603,7 @@
       </c>
       <c r="V110" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9675,7 +9675,7 @@
       </c>
       <c r="V111" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9747,7 +9747,7 @@
       </c>
       <c r="V112" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9819,7 +9819,7 @@
       </c>
       <c r="V113" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9891,7 +9891,7 @@
       </c>
       <c r="V114" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -9963,7 +9963,7 @@
       </c>
       <c r="V115" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -10035,7 +10035,7 @@
       </c>
       <c r="V116" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -10107,7 +10107,7 @@
       </c>
       <c r="V117" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -10179,7 +10179,7 @@
       </c>
       <c r="V118" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -10217,7 +10217,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="K119" t="n">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="V119" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -10323,7 +10323,7 @@
       </c>
       <c r="V120" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -10361,7 +10361,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="K121" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="V121" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -10467,7 +10467,7 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -10539,7 +10539,7 @@
       </c>
       <c r="V123" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
     </row>
@@ -10611,7 +10611,7 @@
       </c>
       <c r="V124" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
     </row>
@@ -10693,28 +10693,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C2" t="n">
-        <v>892</v>
+        <v>791.5</v>
       </c>
       <c r="D2" t="n">
-        <v>928.5</v>
+        <v>801</v>
       </c>
       <c r="E2" t="n">
-        <v>-36.5</v>
+        <v>-9.5</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.03931071620893915</v>
+        <v>-0.0118601747815231</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8119912850729776</v>
+        <v>0.7434118850066025</v>
       </c>
       <c r="H2" t="n">
-        <v>1.398664633453733</v>
+        <v>1.252380169397706</v>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -10730,22 +10730,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>1368</v>
+        <v>1323.5</v>
       </c>
       <c r="D3" t="n">
-        <v>1299.5</v>
+        <v>1278.5</v>
       </c>
       <c r="E3" t="n">
-        <v>68.5</v>
+        <v>45</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05271258176221624</v>
+        <v>0.03519749706687524</v>
       </c>
       <c r="G3" t="n">
-        <v>1.002150741572589</v>
+        <v>1.015003559605596</v>
       </c>
       <c r="H3" t="n">
         <v>1.718757380328138</v>
@@ -10767,25 +10767,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C4" t="n">
-        <v>1694.5</v>
+        <v>2191</v>
       </c>
       <c r="D4" t="n">
-        <v>1699</v>
+        <v>2181</v>
       </c>
       <c r="E4" t="n">
-        <v>-4.5</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.00264861683343143</v>
+        <v>0.004585052728106373</v>
       </c>
       <c r="G4" t="n">
-        <v>0.991851716356334</v>
+        <v>1.031457457846761</v>
       </c>
       <c r="H4" t="n">
-        <v>2.188098591657161</v>
+        <v>2.045654077098847</v>
       </c>
       <c r="I4" t="n">
         <v>6</v>
@@ -10804,28 +10804,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>1939.5</v>
+        <v>1588</v>
       </c>
       <c r="D5" t="n">
-        <v>1873</v>
+        <v>1539.5</v>
       </c>
       <c r="E5" t="n">
-        <v>66.5</v>
+        <v>48.5</v>
       </c>
       <c r="F5" t="n">
-        <v>0.03550453817405232</v>
+        <v>0.03150373497888925</v>
       </c>
       <c r="G5" t="n">
-        <v>1.422424806481158</v>
+        <v>1.456661719659225</v>
       </c>
       <c r="H5" t="n">
         <v>2.682828520472515</v>
       </c>
       <c r="I5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -22618,7 +22618,7 @@
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr">
@@ -22643,7 +22643,7 @@
       </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
@@ -22826,7 +22826,7 @@
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
@@ -22851,7 +22851,7 @@
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
@@ -23035,7 +23035,7 @@
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
@@ -23060,7 +23060,7 @@
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
@@ -23240,7 +23240,7 @@
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como CARVAJAL.</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
@@ -23446,7 +23446,7 @@
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
@@ -23471,7 +23471,7 @@
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
@@ -23672,7 +23672,7 @@
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV7" t="inlineStr">
@@ -23852,7 +23852,7 @@
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
@@ -23877,7 +23877,7 @@
       </c>
       <c r="AU8" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV8" t="inlineStr">
@@ -24057,7 +24057,7 @@
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ9" t="inlineStr">
@@ -24082,7 +24082,7 @@
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV9" t="inlineStr">
@@ -24263,7 +24263,7 @@
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
@@ -24288,7 +24288,7 @@
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV10" t="inlineStr">
@@ -24462,7 +24462,7 @@
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
@@ -24487,7 +24487,7 @@
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
@@ -24667,7 +24667,7 @@
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
@@ -24692,7 +24692,7 @@
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
@@ -24867,7 +24867,7 @@
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>PATIO BONITO</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO13" t="n">
@@ -24875,7 +24875,7 @@
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: PATIO BONITO.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
@@ -24890,17 +24890,17 @@
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>PATIO BONITO</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
@@ -25084,7 +25084,7 @@
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr">
@@ -25109,7 +25109,7 @@
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
@@ -25283,7 +25283,7 @@
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
@@ -25308,7 +25308,7 @@
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV15" t="inlineStr">
@@ -25488,7 +25488,7 @@
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">
@@ -25691,7 +25691,7 @@
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
@@ -25716,7 +25716,7 @@
       </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
@@ -25892,7 +25892,7 @@
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
@@ -25917,7 +25917,7 @@
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
@@ -26097,7 +26097,7 @@
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ19" t="inlineStr">
@@ -26122,7 +26122,7 @@
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
@@ -26288,7 +26288,7 @@
       </c>
       <c r="AN20" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO20" t="n">
@@ -26296,7 +26296,7 @@
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ20" t="inlineStr">
@@ -26311,17 +26311,17 @@
       </c>
       <c r="AS20" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT20" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU20" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV20" t="inlineStr">
@@ -26495,7 +26495,7 @@
       </c>
       <c r="AP21" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ21" t="inlineStr">
@@ -26520,7 +26520,7 @@
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV21" t="inlineStr">
@@ -26700,7 +26700,7 @@
       </c>
       <c r="AP22" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ22" t="inlineStr">
@@ -26725,7 +26725,7 @@
       </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
@@ -26906,7 +26906,7 @@
       </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ23" t="inlineStr">
@@ -26931,7 +26931,7 @@
       </c>
       <c r="AU23" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV23" t="inlineStr">
@@ -27105,7 +27105,7 @@
       </c>
       <c r="AP24" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ24" t="inlineStr">
@@ -27130,7 +27130,7 @@
       </c>
       <c r="AU24" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV24" t="inlineStr">
@@ -27304,7 +27304,7 @@
       </c>
       <c r="AP25" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ25" t="inlineStr">
@@ -27329,7 +27329,7 @@
       </c>
       <c r="AU25" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV25" t="inlineStr">
@@ -27495,7 +27495,7 @@
       </c>
       <c r="AN26" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CLASS ROMA</t>
         </is>
       </c>
       <c r="AO26" t="n">
@@ -27503,7 +27503,7 @@
       </c>
       <c r="AP26" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ26" t="inlineStr">
@@ -27518,17 +27518,17 @@
       </c>
       <c r="AS26" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CLASS ROMA</t>
         </is>
       </c>
       <c r="AT26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU26" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV26" t="inlineStr">
@@ -27708,7 +27708,7 @@
       </c>
       <c r="AP27" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ27" t="inlineStr">
@@ -27733,7 +27733,7 @@
       </c>
       <c r="AU27" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV27" t="inlineStr">
@@ -27907,7 +27907,7 @@
       </c>
       <c r="AP28" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ28" t="inlineStr">
@@ -27932,7 +27932,7 @@
       </c>
       <c r="AU28" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV28" t="inlineStr">
@@ -28113,7 +28113,7 @@
       </c>
       <c r="AP29" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ29" t="inlineStr">
@@ -28138,7 +28138,7 @@
       </c>
       <c r="AU29" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV29" t="inlineStr">
@@ -28312,7 +28312,7 @@
       </c>
       <c r="AP30" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ30" t="inlineStr">
@@ -28337,7 +28337,7 @@
       </c>
       <c r="AU30" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV30" t="inlineStr">
@@ -28503,7 +28503,7 @@
       </c>
       <c r="AN31" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO31" t="n">
@@ -28511,7 +28511,7 @@
       </c>
       <c r="AP31" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ31" t="inlineStr">
@@ -28526,17 +28526,17 @@
       </c>
       <c r="AS31" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT31" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU31" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV31" t="inlineStr">
@@ -28708,7 +28708,7 @@
       </c>
       <c r="AN32" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="AO32" t="n">
@@ -28716,7 +28716,7 @@
       </c>
       <c r="AP32" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ32" t="inlineStr">
@@ -28731,17 +28731,17 @@
       </c>
       <c r="AS32" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="AT32" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU32" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV32" t="inlineStr">
@@ -28907,7 +28907,7 @@
       </c>
       <c r="AN33" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO33" t="n">
@@ -28915,7 +28915,7 @@
       </c>
       <c r="AP33" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ33" t="inlineStr">
@@ -28930,17 +28930,17 @@
       </c>
       <c r="AS33" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT33" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU33" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV33" t="inlineStr">
@@ -29114,7 +29114,7 @@
       </c>
       <c r="AP34" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ34" t="inlineStr">
@@ -29139,7 +29139,7 @@
       </c>
       <c r="AU34" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV34" t="inlineStr">
@@ -29320,7 +29320,7 @@
       </c>
       <c r="AP35" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ35" t="inlineStr">
@@ -29345,7 +29345,7 @@
       </c>
       <c r="AU35" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV35" t="inlineStr">
@@ -29519,7 +29519,7 @@
       </c>
       <c r="AP36" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ36" t="inlineStr">
@@ -29544,7 +29544,7 @@
       </c>
       <c r="AU36" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV36" t="inlineStr">
@@ -29718,7 +29718,7 @@
       </c>
       <c r="AP37" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ37" t="inlineStr">
@@ -29743,7 +29743,7 @@
       </c>
       <c r="AU37" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV37" t="inlineStr">
@@ -29917,7 +29917,7 @@
       </c>
       <c r="AP38" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ38" t="inlineStr">
@@ -29942,7 +29942,7 @@
       </c>
       <c r="AU38" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV38" t="inlineStr">
@@ -30116,7 +30116,7 @@
       </c>
       <c r="AP39" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ39" t="inlineStr">
@@ -30141,7 +30141,7 @@
       </c>
       <c r="AU39" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV39" t="inlineStr">
@@ -30315,7 +30315,7 @@
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ40" t="inlineStr">
@@ -30340,7 +30340,7 @@
       </c>
       <c r="AU40" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV40" t="inlineStr">
@@ -30514,7 +30514,7 @@
       </c>
       <c r="AP41" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ41" t="inlineStr">
@@ -30539,7 +30539,7 @@
       </c>
       <c r="AU41" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV41" t="inlineStr">
@@ -30713,7 +30713,7 @@
       </c>
       <c r="AP42" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ42" t="inlineStr">
@@ -30738,7 +30738,7 @@
       </c>
       <c r="AU42" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV42" t="inlineStr">
@@ -30912,7 +30912,7 @@
       </c>
       <c r="AP43" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ43" t="inlineStr">
@@ -30937,7 +30937,7 @@
       </c>
       <c r="AU43" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV43" t="inlineStr">
@@ -31118,7 +31118,7 @@
       </c>
       <c r="AP44" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
       <c r="AQ44" t="inlineStr">
@@ -31143,7 +31143,7 @@
       </c>
       <c r="AU44" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV44" t="inlineStr">
@@ -31309,7 +31309,7 @@
       </c>
       <c r="AN45" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO45" t="n">
@@ -31317,7 +31317,7 @@
       </c>
       <c r="AP45" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ45" t="inlineStr">
@@ -31332,17 +31332,17 @@
       </c>
       <c r="AS45" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT45" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU45" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV45" t="inlineStr">
@@ -31516,7 +31516,7 @@
       </c>
       <c r="AP46" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ46" t="inlineStr">
@@ -31541,7 +31541,7 @@
       </c>
       <c r="AU46" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV46" t="inlineStr">
@@ -31715,7 +31715,7 @@
       </c>
       <c r="AP47" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ47" t="inlineStr">
@@ -31740,7 +31740,7 @@
       </c>
       <c r="AU47" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV47" t="inlineStr">
@@ -31920,7 +31920,7 @@
       </c>
       <c r="AP48" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ48" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="AU48" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV48" t="inlineStr">
@@ -32119,7 +32119,7 @@
       </c>
       <c r="AP49" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ49" t="inlineStr">
@@ -32144,7 +32144,7 @@
       </c>
       <c r="AU49" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV49" t="inlineStr">
@@ -32318,7 +32318,7 @@
       </c>
       <c r="AP50" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ50" t="inlineStr">
@@ -32343,7 +32343,7 @@
       </c>
       <c r="AU50" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV50" t="inlineStr">
@@ -32517,7 +32517,7 @@
       </c>
       <c r="AP51" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ51" t="inlineStr">
@@ -32542,7 +32542,7 @@
       </c>
       <c r="AU51" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV51" t="inlineStr">
@@ -32723,7 +32723,7 @@
       </c>
       <c r="AP52" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ52" t="inlineStr">
@@ -32748,7 +32748,7 @@
       </c>
       <c r="AU52" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV52" t="inlineStr">
@@ -32928,7 +32928,7 @@
       </c>
       <c r="AP53" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ53" t="inlineStr">
@@ -32953,7 +32953,7 @@
       </c>
       <c r="AU53" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV53" t="inlineStr">
@@ -33127,7 +33127,7 @@
       </c>
       <c r="AP54" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ54" t="inlineStr">
@@ -33152,7 +33152,7 @@
       </c>
       <c r="AU54" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV54" t="inlineStr">
@@ -33326,7 +33326,7 @@
       </c>
       <c r="AP55" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ55" t="inlineStr">
@@ -33351,7 +33351,7 @@
       </c>
       <c r="AU55" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV55" t="inlineStr">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="AP56" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ56" t="inlineStr">
@@ -33550,7 +33550,7 @@
       </c>
       <c r="AU56" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV56" t="inlineStr">
@@ -33724,7 +33724,7 @@
       </c>
       <c r="AP57" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ57" t="inlineStr">
@@ -33749,7 +33749,7 @@
       </c>
       <c r="AU57" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV57" t="inlineStr">
@@ -33929,7 +33929,7 @@
       </c>
       <c r="AP58" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ58" t="inlineStr">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="AU58" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV58" t="inlineStr">
@@ -34127,7 +34127,7 @@
       </c>
       <c r="AN59" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO59" t="n">
@@ -34135,7 +34135,7 @@
       </c>
       <c r="AP59" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ59" t="inlineStr">
@@ -34150,17 +34150,17 @@
       </c>
       <c r="AS59" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT59" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU59" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV59" t="inlineStr">
@@ -34338,7 +34338,7 @@
       </c>
       <c r="AP60" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ60" t="inlineStr">
@@ -34363,7 +34363,7 @@
       </c>
       <c r="AU60" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV60" t="inlineStr">
@@ -34529,7 +34529,7 @@
       </c>
       <c r="AN61" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO61" t="n">
@@ -34537,7 +34537,7 @@
       </c>
       <c r="AP61" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ61" t="inlineStr">
@@ -34552,17 +34552,17 @@
       </c>
       <c r="AS61" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT61" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU61" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV61" t="inlineStr">
@@ -34740,7 +34740,7 @@
       </c>
       <c r="AP62" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ62" t="inlineStr">
@@ -34765,7 +34765,7 @@
       </c>
       <c r="AU62" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV62" t="inlineStr">
@@ -34939,7 +34939,7 @@
       </c>
       <c r="AP63" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ63" t="inlineStr">
@@ -34964,7 +34964,7 @@
       </c>
       <c r="AU63" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV63" t="inlineStr">
@@ -35130,7 +35130,7 @@
       </c>
       <c r="AN64" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO64" t="n">
@@ -35138,7 +35138,7 @@
       </c>
       <c r="AP64" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ64" t="inlineStr">
@@ -35153,17 +35153,17 @@
       </c>
       <c r="AS64" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT64" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU64" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV64" t="inlineStr">
@@ -35329,7 +35329,7 @@
       </c>
       <c r="AN65" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO65" t="n">
@@ -35337,7 +35337,7 @@
       </c>
       <c r="AP65" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ65" t="inlineStr">
@@ -35352,17 +35352,17 @@
       </c>
       <c r="AS65" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT65" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU65" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV65" t="inlineStr">
@@ -35540,7 +35540,7 @@
       </c>
       <c r="AP66" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ66" t="inlineStr">
@@ -35565,7 +35565,7 @@
       </c>
       <c r="AU66" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV66" t="inlineStr">
@@ -35739,7 +35739,7 @@
       </c>
       <c r="AP67" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ67" t="inlineStr">
@@ -35764,7 +35764,7 @@
       </c>
       <c r="AU67" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV67" t="inlineStr">
@@ -35938,7 +35938,7 @@
       </c>
       <c r="AP68" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ68" t="inlineStr">
@@ -35963,7 +35963,7 @@
       </c>
       <c r="AU68" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV68" t="inlineStr">
@@ -36137,7 +36137,7 @@
       </c>
       <c r="AP69" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ69" t="inlineStr">
@@ -36162,7 +36162,7 @@
       </c>
       <c r="AU69" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV69" t="inlineStr">
@@ -36336,7 +36336,7 @@
       </c>
       <c r="AP70" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ70" t="inlineStr">
@@ -36361,7 +36361,7 @@
       </c>
       <c r="AU70" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV70" t="inlineStr">
@@ -36535,7 +36535,7 @@
       </c>
       <c r="AP71" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
       <c r="AQ71" t="inlineStr">
@@ -36560,7 +36560,7 @@
       </c>
       <c r="AU71" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV71" t="inlineStr">
@@ -36734,7 +36734,7 @@
       </c>
       <c r="AP72" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ72" t="inlineStr">
@@ -36759,7 +36759,7 @@
       </c>
       <c r="AU72" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV72" t="inlineStr">
@@ -36941,7 +36941,7 @@
       </c>
       <c r="AP73" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ73" t="inlineStr">
@@ -36966,7 +36966,7 @@
       </c>
       <c r="AU73" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV73" t="inlineStr">
@@ -37144,7 +37144,7 @@
       </c>
       <c r="AP74" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ74" t="inlineStr">
@@ -37169,7 +37169,7 @@
       </c>
       <c r="AU74" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV74" t="inlineStr">
@@ -37343,7 +37343,7 @@
       </c>
       <c r="AP75" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ75" t="inlineStr">
@@ -37368,7 +37368,7 @@
       </c>
       <c r="AU75" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV75" t="inlineStr">
@@ -37542,7 +37542,7 @@
       </c>
       <c r="AP76" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
       <c r="AQ76" t="inlineStr">
@@ -37567,7 +37567,7 @@
       </c>
       <c r="AU76" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV76" t="inlineStr">
@@ -37741,7 +37741,7 @@
       </c>
       <c r="AP77" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ77" t="inlineStr">
@@ -37766,7 +37766,7 @@
       </c>
       <c r="AU77" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV77" t="inlineStr">
@@ -37944,7 +37944,7 @@
       </c>
       <c r="AP78" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
       <c r="AQ78" t="inlineStr">
@@ -37969,7 +37969,7 @@
       </c>
       <c r="AU78" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV78" t="inlineStr">
@@ -38143,7 +38143,7 @@
       </c>
       <c r="AP79" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ79" t="inlineStr">
@@ -38168,7 +38168,7 @@
       </c>
       <c r="AU79" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV79" t="inlineStr">
@@ -38338,7 +38338,7 @@
       </c>
       <c r="AN80" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="AO80" t="n">
@@ -38346,7 +38346,7 @@
       </c>
       <c r="AP80" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ80" t="inlineStr">
@@ -38361,17 +38361,17 @@
       </c>
       <c r="AS80" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="AT80" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU80" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV80" t="inlineStr">
@@ -38545,7 +38545,7 @@
       </c>
       <c r="AP81" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ81" t="inlineStr">
@@ -38570,7 +38570,7 @@
       </c>
       <c r="AU81" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV81" t="inlineStr">
@@ -38750,7 +38750,7 @@
       </c>
       <c r="AP82" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ82" t="inlineStr">
@@ -38775,7 +38775,7 @@
       </c>
       <c r="AU82" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV82" t="inlineStr">
@@ -38949,7 +38949,7 @@
       </c>
       <c r="AP83" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ83" t="inlineStr">
@@ -38974,7 +38974,7 @@
       </c>
       <c r="AU83" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV83" t="inlineStr">
@@ -39156,7 +39156,7 @@
       </c>
       <c r="AP84" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ84" t="inlineStr">
@@ -39181,7 +39181,7 @@
       </c>
       <c r="AU84" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV84" t="inlineStr">
@@ -39355,7 +39355,7 @@
       </c>
       <c r="AP85" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ85" t="inlineStr">
@@ -39380,7 +39380,7 @@
       </c>
       <c r="AU85" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV85" t="inlineStr">
@@ -39554,7 +39554,7 @@
       </c>
       <c r="AP86" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ86" t="inlineStr">
@@ -39579,7 +39579,7 @@
       </c>
       <c r="AU86" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV86" t="inlineStr">
@@ -39753,7 +39753,7 @@
       </c>
       <c r="AP87" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ87" t="inlineStr">
@@ -39778,7 +39778,7 @@
       </c>
       <c r="AU87" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV87" t="inlineStr">
@@ -39944,7 +39944,7 @@
       </c>
       <c r="AN88" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="AO88" t="n">
@@ -39952,7 +39952,7 @@
       </c>
       <c r="AP88" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: KENNEDY CENTRAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ88" t="inlineStr">
@@ -39967,17 +39967,17 @@
       </c>
       <c r="AS88" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="AT88" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU88" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV88" t="inlineStr">
@@ -40151,7 +40151,7 @@
       </c>
       <c r="AP89" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ89" t="inlineStr">
@@ -40176,7 +40176,7 @@
       </c>
       <c r="AU89" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV89" t="inlineStr">
@@ -40350,7 +40350,7 @@
       </c>
       <c r="AP90" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ90" t="inlineStr">
@@ -40375,7 +40375,7 @@
       </c>
       <c r="AU90" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV90" t="inlineStr">
@@ -40549,7 +40549,7 @@
       </c>
       <c r="AP91" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ91" t="inlineStr">
@@ -40574,7 +40574,7 @@
       </c>
       <c r="AU91" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV91" t="inlineStr">
@@ -40752,7 +40752,7 @@
       </c>
       <c r="AP92" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ92" t="inlineStr">
@@ -40777,7 +40777,7 @@
       </c>
       <c r="AU92" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV92" t="inlineStr">
@@ -40951,7 +40951,7 @@
       </c>
       <c r="AP93" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ93" t="inlineStr">
@@ -40976,7 +40976,7 @@
       </c>
       <c r="AU93" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV93" t="inlineStr">
@@ -41150,7 +41150,7 @@
       </c>
       <c r="AP94" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ94" t="inlineStr">
@@ -41175,7 +41175,7 @@
       </c>
       <c r="AU94" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV94" t="inlineStr">
@@ -41353,7 +41353,7 @@
       </c>
       <c r="AP95" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ95" t="inlineStr">
@@ -41378,7 +41378,7 @@
       </c>
       <c r="AU95" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV95" t="inlineStr">
@@ -41544,7 +41544,7 @@
       </c>
       <c r="AN96" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO96" t="n">
@@ -41552,7 +41552,7 @@
       </c>
       <c r="AP96" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ96" t="inlineStr">
@@ -41567,17 +41567,17 @@
       </c>
       <c r="AS96" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT96" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU96" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV96" t="inlineStr">
@@ -41751,7 +41751,7 @@
       </c>
       <c r="AP97" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ97" t="inlineStr">
@@ -41776,7 +41776,7 @@
       </c>
       <c r="AU97" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV97" t="inlineStr">
@@ -41942,7 +41942,7 @@
       </c>
       <c r="AN98" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO98" t="n">
@@ -41950,7 +41950,7 @@
       </c>
       <c r="AP98" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ98" t="inlineStr">
@@ -41965,17 +41965,17 @@
       </c>
       <c r="AS98" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT98" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU98" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV98" t="inlineStr">
@@ -42153,7 +42153,7 @@
       </c>
       <c r="AP99" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ99" t="inlineStr">
@@ -42178,7 +42178,7 @@
       </c>
       <c r="AU99" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV99" t="inlineStr">
@@ -42352,7 +42352,7 @@
       </c>
       <c r="AP100" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como PATIO BONITO.</t>
         </is>
       </c>
       <c r="AQ100" t="inlineStr">
@@ -42377,7 +42377,7 @@
       </c>
       <c r="AU100" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV100" t="inlineStr">
@@ -42555,7 +42555,7 @@
       </c>
       <c r="AP101" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ101" t="inlineStr">
@@ -42580,7 +42580,7 @@
       </c>
       <c r="AU101" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV101" t="inlineStr">
@@ -42754,7 +42754,7 @@
       </c>
       <c r="AP102" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ102" t="inlineStr">
@@ -42779,7 +42779,7 @@
       </c>
       <c r="AU102" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV102" t="inlineStr">
@@ -42953,7 +42953,7 @@
       </c>
       <c r="AP103" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ103" t="inlineStr">
@@ -42978,7 +42978,7 @@
       </c>
       <c r="AU103" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV103" t="inlineStr">
@@ -43156,7 +43156,7 @@
       </c>
       <c r="AP104" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ104" t="inlineStr">
@@ -43181,7 +43181,7 @@
       </c>
       <c r="AU104" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV104" t="inlineStr">
@@ -43355,7 +43355,7 @@
       </c>
       <c r="AP105" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ105" t="inlineStr">
@@ -43380,7 +43380,7 @@
       </c>
       <c r="AU105" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV105" t="inlineStr">
@@ -43554,7 +43554,7 @@
       </c>
       <c r="AP106" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ106" t="inlineStr">
@@ -43579,7 +43579,7 @@
       </c>
       <c r="AU106" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV106" t="inlineStr">
@@ -43757,7 +43757,7 @@
       </c>
       <c r="AP107" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ107" t="inlineStr">
@@ -43782,7 +43782,7 @@
       </c>
       <c r="AU107" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV107" t="inlineStr">
@@ -43960,7 +43960,7 @@
       </c>
       <c r="AP108" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ108" t="inlineStr">
@@ -43985,7 +43985,7 @@
       </c>
       <c r="AU108" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV108" t="inlineStr">
@@ -44159,7 +44159,7 @@
       </c>
       <c r="AP109" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ109" t="inlineStr">
@@ -44184,7 +44184,7 @@
       </c>
       <c r="AU109" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV109" t="inlineStr">
@@ -44358,7 +44358,7 @@
       </c>
       <c r="AP110" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ110" t="inlineStr">
@@ -44383,7 +44383,7 @@
       </c>
       <c r="AU110" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV110" t="inlineStr">
@@ -44543,7 +44543,7 @@
       </c>
       <c r="AP111" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ111" t="inlineStr">
@@ -44568,7 +44568,7 @@
       </c>
       <c r="AU111" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV111" t="inlineStr">
@@ -44728,7 +44728,7 @@
       </c>
       <c r="AP112" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ112" t="inlineStr">
@@ -44753,7 +44753,7 @@
       </c>
       <c r="AU112" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV112" t="inlineStr">
@@ -44913,7 +44913,7 @@
       </c>
       <c r="AP113" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ113" t="inlineStr">
@@ -44938,7 +44938,7 @@
       </c>
       <c r="AU113" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV113" t="inlineStr">
@@ -45098,7 +45098,7 @@
       </c>
       <c r="AP114" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ114" t="inlineStr">
@@ -45123,7 +45123,7 @@
       </c>
       <c r="AU114" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV114" t="inlineStr">
@@ -45283,7 +45283,7 @@
       </c>
       <c r="AP115" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ115" t="inlineStr">
@@ -45308,7 +45308,7 @@
       </c>
       <c r="AU115" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV115" t="inlineStr">
@@ -45468,7 +45468,7 @@
       </c>
       <c r="AP116" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ116" t="inlineStr">
@@ -45493,7 +45493,7 @@
       </c>
       <c r="AU116" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV116" t="inlineStr">
@@ -45653,7 +45653,7 @@
       </c>
       <c r="AP117" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ117" t="inlineStr">
@@ -45678,7 +45678,7 @@
       </c>
       <c r="AU117" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV117" t="inlineStr">
@@ -45838,7 +45838,7 @@
       </c>
       <c r="AP118" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ118" t="inlineStr">
@@ -45863,7 +45863,7 @@
       </c>
       <c r="AU118" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV118" t="inlineStr">
@@ -46015,7 +46015,7 @@
       </c>
       <c r="AN119" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="AO119" t="n">
@@ -46023,7 +46023,7 @@
       </c>
       <c r="AP119" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CLASS ROMA.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ119" t="inlineStr">
@@ -46038,17 +46038,17 @@
       </c>
       <c r="AS119" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="AT119" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU119" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV119" t="inlineStr">
@@ -46208,7 +46208,7 @@
       </c>
       <c r="AP120" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ120" t="inlineStr">
@@ -46233,7 +46233,7 @@
       </c>
       <c r="AU120" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV120" t="inlineStr">
@@ -46385,7 +46385,7 @@
       </c>
       <c r="AN121" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AO121" t="n">
@@ -46393,7 +46393,7 @@
       </c>
       <c r="AP121" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: CARVAJAL.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ121" t="inlineStr">
@@ -46408,17 +46408,17 @@
       </c>
       <c r="AS121" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="AT121" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AU121" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV121" t="inlineStr">
@@ -46578,7 +46578,7 @@
       </c>
       <c r="AP122" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ122" t="inlineStr">
@@ -46603,7 +46603,7 @@
       </c>
       <c r="AU122" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV122" t="inlineStr">
@@ -46763,7 +46763,7 @@
       </c>
       <c r="AP123" t="inlineStr">
         <is>
-          <t>Coincide con iglesia actual.</t>
+          <t>Se conserva el templo asignado en el documento base.</t>
         </is>
       </c>
       <c r="AQ123" t="inlineStr">
@@ -46788,7 +46788,7 @@
       </c>
       <c r="AU123" t="inlineStr">
         <is>
-          <t>La asignación propuesta coincide con la iglesia histórica 2026.</t>
+          <t>Se conserva la asignación documental del puesto.</t>
         </is>
       </c>
       <c r="AV123" t="inlineStr">
@@ -46948,7 +46948,7 @@
       </c>
       <c r="AP124" t="inlineStr">
         <is>
-          <t>Reasignación sugerida por cercanía: VALLADOLID.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; la asignación documental se mantiene como KENNEDY CENTRAL.</t>
         </is>
       </c>
       <c r="AQ124" t="inlineStr">
@@ -46973,7 +46973,7 @@
       </c>
       <c r="AU124" t="inlineStr">
         <is>
-          <t>Asignación sugerida por cercanía territorial; conserva iglesia histórica para análisis electoral.</t>
+          <t>Propuesta específica para Valladolid por cercanía territorial; los demás templos conservan la asignación documental.</t>
         </is>
       </c>
       <c r="AV124" t="inlineStr">
@@ -65677,12 +65677,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PATIO BONITO</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -66202,12 +66202,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -66652,12 +66652,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CLASS ROMA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -67027,12 +67027,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -67102,12 +67102,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -67177,12 +67177,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -68077,12 +68077,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -69127,12 +69127,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -69277,12 +69277,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -69502,12 +69502,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -69577,12 +69577,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -70702,12 +70702,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -71302,12 +71302,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -71902,12 +71902,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -72052,12 +72052,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -73579,12 +73579,12 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -73717,12 +73717,12 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -75342,12 +75342,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>PATIO BONITO</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -75391,7 +75391,7 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>PATIO BONITO</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -75965,12 +75965,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -76014,7 +76014,7 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -76499,12 +76499,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CLASS ROMA</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -76548,7 +76548,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CLASS ROMA</t>
         </is>
       </c>
     </row>
@@ -76944,12 +76944,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -76993,7 +76993,7 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -77033,12 +77033,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -77082,7 +77082,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
     </row>
@@ -77122,12 +77122,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -77171,7 +77171,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -78190,12 +78190,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
@@ -78239,7 +78239,7 @@
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -79436,12 +79436,12 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J59" t="inlineStr"/>
@@ -79485,7 +79485,7 @@
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -79614,12 +79614,12 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J61" t="inlineStr"/>
@@ -79663,7 +79663,7 @@
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -79881,12 +79881,12 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J64" t="inlineStr"/>
@@ -79930,7 +79930,7 @@
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -79970,12 +79970,12 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J65" t="inlineStr"/>
@@ -80019,7 +80019,7 @@
       </c>
       <c r="U65" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -81305,12 +81305,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J80" t="inlineStr"/>
@@ -81354,7 +81354,7 @@
       </c>
       <c r="U80" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
     </row>
@@ -82017,12 +82017,12 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J88" t="inlineStr"/>
@@ -82066,7 +82066,7 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>KENNEDY CENTRAL</t>
+          <t>PATIO BONITO</t>
         </is>
       </c>
     </row>
@@ -82729,12 +82729,12 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J96" t="inlineStr"/>
@@ -82778,7 +82778,7 @@
       </c>
       <c r="U96" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -82907,12 +82907,12 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J98" t="inlineStr"/>
@@ -82956,7 +82956,7 @@
       </c>
       <c r="U98" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>
@@ -84728,12 +84728,12 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J119" t="inlineStr"/>
@@ -84771,7 +84771,7 @@
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>CLASS ROMA</t>
+          <t>CARVAJAL</t>
         </is>
       </c>
     </row>
@@ -84894,12 +84894,12 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J121" t="inlineStr"/>
@@ -84937,7 +84937,7 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>CARVAJAL</t>
+          <t>KENNEDY CENTRAL</t>
         </is>
       </c>
     </row>

</xml_diff>